<commit_message>
Add Sehore LULC ESRI 10m Statistics Excel file and update TIF File Inventory
</commit_message>
<xml_diff>
--- a/Sehore_TIF_File_Inventory.xlsx
+++ b/Sehore_TIF_File_Inventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Epics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_093DEF541FB4723BF4CE5A5ADF7644CDDFF369B4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDA45A3-E422-49E7-A4E9-CF03E82610DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,16 +16,11 @@
     <sheet name="TIF File Inventory" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="77">
   <si>
     <t>File Name</t>
   </si>
@@ -229,25 +224,45 @@
   </si>
   <si>
     <t>Sehore_Water_NDWI_2024.tif</t>
+  </si>
+  <si>
+    <t>Sehore_LULC_10m_2017.tif</t>
+  </si>
+  <si>
+    <t>Land Use/Land Cover classification (Impact Observatory/ESRI Sentinel-2-derived ML scheme, remapped into the same Forest/Grass-Savanna/Wetland/Cropland/Urban/Barren/Water categories as the MODIS layer), 2017. 10m resolution — a 2,500x pixel-count improvement over the 500m MODIS version, and now the primary LULC layer for the report. IMPORTANT: contradicts MODIS on Forest trend direction (MODIS shows forest increasing, ESRI shows it declining) — see Sehore_LULC_ESRI_10m_Statistics.xlsx for the full comparison and explanation.</t>
+  </si>
+  <si>
+    <t>ESRI/Impact Observatory Global-LULC 10m Time Series, via Sentinel-2</t>
+  </si>
+  <si>
+    <t>03_LULC_Statistics_ESRI_10m.js</t>
+  </si>
+  <si>
+    <t>Sehore_LULC_10m_2020.tif</t>
+  </si>
+  <si>
+    <t>Same as above, for 2020.</t>
+  </si>
+  <si>
+    <t>Sehore_LULC_10m_Change_2017_2020.tif</t>
+  </si>
+  <si>
+    <t>Binary change layer (1 = category changed, 0 = no change) between the 2017 and 2020 ESRI 10m classifications — the high-resolution equivalent of the MODIS-based change layer.</t>
+  </si>
+  <si>
+    <t>Derived from ESRI/Impact Observatory 10m LULC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
       <charset val="1"/>
     </font>
     <font>
@@ -266,6 +281,19 @@
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -309,28 +337,80 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFD9D9D9"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border outline="0">
+        <right style="thin">
+          <color rgb="FFD9D9D9"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Times New Roman"/>
+        <family val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -412,15 +492,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TIFInventory" displayName="TIFInventory" ref="A1:F19" totalsRowShown="0">
-  <autoFilter ref="A1:F19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="TIFInventory" displayName="TIFInventory" ref="A1:F22" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A1:F22" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="File Name"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Folder"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Data Source / Satellite"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Resolution"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Generated By"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="File Name" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Folder" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Description" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Data Source / Satellite" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Resolution" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Generated By" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -605,395 +685,456 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="62" customWidth="1"/>
-    <col min="4" max="4" width="24" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="1" max="1" width="43.5546875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="20" style="7" customWidth="1"/>
+    <col min="3" max="3" width="62" style="7" customWidth="1"/>
+    <col min="4" max="4" width="24" style="7" customWidth="1"/>
+    <col min="5" max="5" width="14" style="7" customWidth="1"/>
+    <col min="6" max="6" width="32" style="7" customWidth="1"/>
+    <col min="7" max="16384" width="8.6640625" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="E3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="E4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="E5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="6" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="6" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="3" t="s">
+      <c r="B10" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="B11" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="B12" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="B13" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="3" t="s">
+      <c r="E13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="3" t="s">
+      <c r="B14" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" s="3" t="s">
+      <c r="E14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="3" t="s">
+      <c r="B15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="3" t="s">
+      <c r="E15" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="B16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" s="3" t="s">
+      <c r="E16" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="B17" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E17" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="3" t="s">
+      <c r="E17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="3" t="s">
+      <c r="B18" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="3" t="s">
+      <c r="E18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="B19" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="E19" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="6" t="s">
         <v>61</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>